<commit_message>
fix(inventory): share sodium-ion capacity learning with stationary storage
Make stationary sodium-ion capacity purchase exactly one kWh of the existing chemistry-specific capacity reference. Its existing cell-density trajectory (157 to200 Wh/kg,2020-2050) then applies once, while module manufacture/end-of-life and fixed auxiliary hardware are no longer duplicated at the stationary wrapper. Module mass changes from8.474582 to6.652547 kg/kWh over that interval. Retain stationary operation/lifetime assumptions and scenario shares. Only the existing capacity workbook changes; no runtime or YAML edits.

Validation: reviewed-candidate equivalence including formula caches; ten ecoinvent3.8-3.12/uncertainty configurations and eight scenario years. Document the shared reference and its assumptions in the existing activity comment.
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-battery-capacity.xlsx
+++ b/premise/data/additional_inventories/lci-battery-capacity.xlsx
@@ -7232,7 +7232,9 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>APPROVED ENGINEERING CONTROL/THERMAL COVERAGE, item13, 2026-10-18. Wickerts corrected SI DOI10.1021/acssuschemeng.4c01782.s001 S26/S27; original Ellingsen2014 SI S39/S40, DOI10.1111/jiec.12072. Separate module monitoring from central protection: per16-module reference,1.1kg populated PCB monitors, central0.49kg populated PCB+2.8kg HV system+1.2kg LV system+.028kg fasteners=4.518kg. Use existing HV/LV/fastener process providers and generic populated through-hole PCB perkg; this is an explicit board-technology/material proxy rather than the source-specific board fabrication model. No whole BMS is added on top. Adopt one nominal10kg liquid-cooling assembly per reference: Al9.08, steel.23, PVC/rubber pipe.0096, thermal pad.2 (silicon.06, glass.02, ABS.12), ethylene glycol.48kg; source-rounded sum9.9996kg. Metal working/injection services are included; 100percent retention of listed finished materials is assumed. No stationary rack housing/container, common vehicle body or roadway is added. Monitoring/protection/cooling are added once as a unit-valued capacity input; kg module and matching waste remain separate, so density learning does not shrink fixed controls. Central and cooling hardware are conservatively co-replaced with each delivered pack; longer independent hardware life is not established. End-of-life uses the existing generic used Li-ion route for15.6176kg of auxiliary hardware per reference, without recovery credits; this is a treatment proxy for controls/cooling, not proof of chemistry-specific recovery. Source thermal duty, pump/radiator performance, protection ratings, inverter/pack interface, full outer pack enclosure and vehicle-specific module topology remain coverage/design gaps. The SIB cell-mass-equivalent module retains its existing18.768kg cell+6.203kg module hardware reference; it is not a demonstrated integer21700-cell topology. LiS uses the corrected19.306152kg cell+6.203kg module hardware. These are engineering references, not fleet-validated designs; use0.5-2x auxiliary-size and independent-replacement-life sensitivities. Reference gross capacity is16*18.768kg cell*0.157kWh/kg=47.145216000000005kWh; dose=0.02121105988781555unit/kWh. Existing cell density, kg-module recipe, energy/per-MJ coefficients and cycle assumptions are preserved.
+          <t>APPROVED STATIONARY SODIUM-ION SHARED CAPACITY REFERENCE, item21,2026-10-18. The stationary NMMT/HC module recipe and baseline specific energy match the existing chemistry-specific capacity reference. Its stationary name is absent from energy_density.yaml, so direct kg inputs stay constant while the common chemistry reference follows157Wh/kg-cell in2020 to200Wh/kg-cell in2050. Preserve workbook-only scope by purchasing exactly1kWh of market for battery capacity,Sodium-ion,SiB atGLO. This existing reference already supplies module manufacturing, equal negative end-of-life mass and the separately fixed-unit monitoring/protection/cooling package. Remove the stationary wrapper duplicate kg-manufacturing, waste and auxiliary inputs; do not add end-of-life twice. The wrapper itself is unmapped and receives no second density adjustment. Original stationary storage operating efficiency, calendar/cycle life and aggregate scenario shares are unchanged; this capacity reference contains manufacture and end-of-life rather than vehicle operation. The cell density trajectory is the existing scenario assumption, not a measured stationary pack design. Expected module mass8.474582023338275kg/kWh in2020 and6.652546888320545kg/kWh in2050, with fixed auxiliary input0.02121105988781555unit/kWh. No runtime or YAML modification.
+PREVIOUS NOTES (retained as history; the correction above takes precedence):
+APPROVED ENGINEERING CONTROL/THERMAL COVERAGE, item13, 2026-10-18. Wickerts corrected SI DOI10.1021/acssuschemeng.4c01782.s001 S26/S27; original Ellingsen2014 SI S39/S40, DOI10.1111/jiec.12072. Separate module monitoring from central protection: per16-module reference,1.1kg populated PCB monitors, central0.49kg populated PCB+2.8kg HV system+1.2kg LV system+.028kg fasteners=4.518kg. Use existing HV/LV/fastener process providers and generic populated through-hole PCB perkg; this is an explicit board-technology/material proxy rather than the source-specific board fabrication model. No whole BMS is added on top. Adopt one nominal10kg liquid-cooling assembly per reference: Al9.08, steel.23, PVC/rubber pipe.0096, thermal pad.2 (silicon.06, glass.02, ABS.12), ethylene glycol.48kg; source-rounded sum9.9996kg. Metal working/injection services are included; 100percent retention of listed finished materials is assumed. No stationary rack housing/container, common vehicle body or roadway is added. Monitoring/protection/cooling are added once as a unit-valued capacity input; kg module and matching waste remain separate, so density learning does not shrink fixed controls. Central and cooling hardware are conservatively co-replaced with each delivered pack; longer independent hardware life is not established. End-of-life uses the existing generic used Li-ion route for15.6176kg of auxiliary hardware per reference, without recovery credits; this is a treatment proxy for controls/cooling, not proof of chemistry-specific recovery. Source thermal duty, pump/radiator performance, protection ratings, inverter/pack interface, full outer pack enclosure and vehicle-specific module topology remain coverage/design gaps. The SIB cell-mass-equivalent module retains its existing18.768kg cell+6.203kg module hardware reference; it is not a demonstrated integer21700-cell topology. LiS uses the corrected19.306152kg cell+6.203kg module hardware. These are engineering references, not fleet-validated designs; use0.5-2x auxiliary-size and independent-replacement-life sensitivities. Reference gross capacity is16*18.768kg cell*0.157kWh/kg=47.145216000000005kWh; dose=0.02121105988781555unit/kWh. Existing cell density, kg-module recipe, energy/per-MJ coefficients and cycle assumptions are preserved.
 PREVIOUS NOTES (retained as history; the correction above takes precedence):
 APPROVED STATIONARY SODIUM-ION CAPACITY BASELINE NORMALIZATION, 2026-10-18. Zhang et al. (2024), Future climate impacts of sodium-ion batteries, Resources, Conservation and Recycling 202, 107362, DOI 10.1016/j.resconrec.2023.107362, Table 4, page 5: baseline NMMT/HC cell specific energy is 157 Wh/kg (0.157 kWh/kg), consistent with the existing source description and Premise density baseline. Primary paper: https://pub.epsilon.slu.se/32553/1/zhang-s-et-al-20240122.pdf . The linked existing SIB module recipe contains 0.7515918465419887 kg NMMT cell/kg module (lci-batteries-SIB.xlsx, sodium-ion batteries B493); its battery market purchases one kg of this module per kg delivered. Use this actual recipe coefficient, not a rounded 75 percent fraction, and 0.157 kWh/kg cell: 1/(0.157*0.7515918465419887) = 8.474582023338275 kg delivered module/kWh gross capacity. The previous 1/(0.16*0.75) = 8.333333333333334 kg represented 0.9833326658924353 kWh under those declared specifications. The module dose increases 1.6949842800592974 percent; this is not a percent change in overall transport or system metal demand. Set battery cell mass share to the linked recipe coefficient. Keep existing cell-specific density uncertainty endpoints 0.12 and 0.18 kWh/kg, translating them with the same module fraction; retain triangular type 5, equal negative waste mass and paired signed bounds/locations. Update formula caches consistently. The original rounded specific-energy/fraction/mass figures below are historical notes superseded by this paragraph. All supplier identities/geographies, the one-kWh output, cell/module manufacturing recipes, other chemistries, prospective density trajectory and lifetime/per-MJ allocations remain unchanged. This normalizes to declared cell energy and an existing module proxy; it does not validate measured pack performance, future electrochemical charge, cycle life or operating conditions. The Li-S-derived module architecture and missing BMS/cooling coverage remain unresolved. No electronics, racks, treatment route, recovery credit or primary/secondary share is added. Current full-system metal effects remain unquantified without a scenario rebuild. STATIONARY MAPPING LIMITATION: This stationary capacity-market name is absent from the existing density aliases. The current unmodified updater therefore leaves its mass and uncertainty bounds fixed through 2050. This corrects the initial normalization only; it does not implement the mobile density trajectory or resolve that mapping gap. The stationary market was inactive in the last 28-case audit, so no current system-metal effect is inferred. The previous mobile correction is preserved.
 PREVIOUS SOURCE NOTES (ROUNDED VALUES SUPERSEDED ABOVE):
@@ -7346,15 +7348,19 @@
       </c>
     </row>
     <row r="118" spans="1:14" ns3:dyDescent="0.2">
-      <c r="A118" t="s">
-        <v>39</v>
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>market for battery capacity, Sodium-ion, SiB</t>
+        </is>
       </c>
       <c r="B118" s="3">
-        <f>1/(0.157*$B$114)</f>
-        <v>8.474582023338275</v>
-      </c>
-      <c r="C118" t="s">
-        <v>7</v>
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>kilowatt hour</t>
+        </is>
       </c>
       <c r="D118" t="s">
         <v>3</v>
@@ -7362,100 +7368,41 @@
       <c r="E118" t="s">
         <v>14</v>
       </c>
-      <c r="F118" t="s">
-        <v>40</v>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>electricity storage capacity</t>
+        </is>
       </c>
       <c r="G118">
-        <v>5</v>
-      </c>
-      <c r="H118" s="7">
-        <f>B118</f>
-        <v>8.474582023338275</v>
-      </c>
-      <c r="I118" s="3">
-        <f>1/(0.18*$B$114)</f>
-        <v>7.391718764800606</v>
-      </c>
-      <c r="J118" s="3">
-        <f>1/(0.12*$B$114)</f>
-        <v>11.08757814720091</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H118" s="7"/>
+      <c r="I118" s="3"/>
+      <c r="J118" s="3"/>
     </row>
     <row r="119" spans="1:14" ns3:dyDescent="0.2">
-      <c r="A119" t="s">
-        <v>53</v>
-      </c>
-      <c r="B119" s="3">
-        <f>-1*B118</f>
-        <v>-8.474582023338275</v>
-      </c>
-      <c r="C119" t="s">
-        <v>7</v>
-      </c>
-      <c r="D119" t="s">
-        <v>3</v>
-      </c>
-      <c r="E119" t="s">
-        <v>14</v>
-      </c>
-      <c r="F119" t="s">
-        <v>54</v>
-      </c>
-      <c r="G119">
-        <v>5</v>
-      </c>
-      <c r="H119" s="7">
-        <f>B119</f>
-        <v>-8.474582023338275</v>
-      </c>
-      <c r="I119" s="3">
-        <f>-1/(0.12*$B$114)</f>
-        <v>-11.08757814720091</v>
-      </c>
-      <c r="J119" s="3">
-        <f>-1/(0.18*$B$114)</f>
-        <v>-7.391718764800606</v>
-      </c>
-      <c r="K119" t="b">
-        <v>1</v>
-      </c>
+      <c r="A119"/>
+      <c r="B119" s="3"/>
+      <c r="C119"/>
+      <c r="D119"/>
+      <c r="E119"/>
+      <c r="F119"/>
+      <c r="G119"/>
+      <c r="H119" s="7"/>
+      <c r="I119" s="3"/>
+      <c r="J119" s="3"/>
+      <c r="K119"/>
       <c r="M119" s="3"/>
       <c r="N119" s="3"/>
     </row>
     <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>battery controls and cooling, 16-module engineering reference</t>
-        </is>
-      </c>
-      <c r="B120">
-        <v>0.02121105988781555</v>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>GLO</t>
-        </is>
-      </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>technosphere</t>
-        </is>
-      </c>
-      <c r="F120" t="inlineStr">
-        <is>
-          <t>battery controls and cooling, 16-module engineering reference</t>
-        </is>
-      </c>
-      <c r="L120" t="inlineStr">
-        <is>
-          <t>Engineering auxiliary input; fixed unit reference, includes own separate15.6176kg waste.</t>
-        </is>
-      </c>
+      <c r="A120"/>
+      <c r="B120"/>
+      <c r="C120"/>
+      <c r="D120"/>
+      <c r="E120"/>
+      <c r="F120"/>
+      <c r="L120"/>
     </row>
     <row r="121" spans="1:14" ht="16" ns3:dyDescent="0.2">
       <c r="A121" s="2" t="s">

</xml_diff>